<commit_message>
& - 86031343 от 13.02.2026 https://meshok.net/
</commit_message>
<xml_diff>
--- a/Collections/Russia/#Russia#Russian_Federation#Regular#[1992-present]#circulation_quality.xlsx
+++ b/Collections/Russia/#Russia#Russian_Federation#Regular#[1992-present]#circulation_quality.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\Russia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D884F74B-5198-46CC-B3D8-402EFC2562E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3E1699-43E1-4CC0-8384-FC4DC74C03AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -828,7 +828,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2293" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2275" uniqueCount="60">
   <si>
     <t>-</t>
   </si>
@@ -1014,7 +1014,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1071,8 +1071,15 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="0.39997558519241921"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1115,8 +1122,14 @@
         <bgColor rgb="FFF2DBDB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1202,13 +1215,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1313,13 +1341,136 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="62">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1336,6 +1487,14 @@
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -2735,9 +2894,9 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="2" dataCellStyle="Гиперссылка"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="17" dataCellStyle="Гиперссылка"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -3985,8 +4144,8 @@
       <c r="G35" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H35" s="21" t="s">
-        <v>0</v>
+      <c r="H35" s="38">
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -4007,8 +4166,8 @@
       <c r="G36" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="21" t="s">
-        <v>0</v>
+      <c r="H36" s="38">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4020,12 +4179,12 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H26">
-    <cfRule type="containsText" dxfId="45" priority="20" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="61" priority="24" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:H26">
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -4037,12 +4196,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="containsText" dxfId="44" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="60" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H28))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="colorScale" priority="10">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -4054,12 +4213,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28">
-    <cfRule type="containsText" dxfId="43" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="59" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G28))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -4071,11 +4230,45 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:H34">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="58" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:H34">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="containsText" dxfId="15" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -5209,7 +5402,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H4">
-    <cfRule type="containsText" dxfId="13" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="28" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -5224,7 +5417,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:H5">
-    <cfRule type="containsText" dxfId="12" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="27" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G5))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -5239,7 +5432,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:H16">
-    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="26" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G6))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -5254,7 +5447,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:H34 G36:H36">
-    <cfRule type="containsText" dxfId="10" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="25" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -5269,7 +5462,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G35:H35 G37:H37">
-    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -6371,7 +6564,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H3">
-    <cfRule type="containsText" dxfId="8" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="23" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -6386,7 +6579,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:H4">
-    <cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="22" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -6401,7 +6594,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:H15">
-    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="21" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G5))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -6416,7 +6609,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G16:H33 G35:H35">
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="20" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6431,7 +6624,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:H34 G36:H36">
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -7501,8 +7694,8 @@
       <c r="G35" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H35" s="21" t="s">
-        <v>0</v>
+      <c r="H35" s="38">
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -7523,8 +7716,8 @@
       <c r="G36" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="21" t="s">
-        <v>0</v>
+      <c r="H36" s="38">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -7536,12 +7729,12 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H26">
-    <cfRule type="containsText" dxfId="42" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="57" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:H26">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -7553,12 +7746,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="containsText" dxfId="41" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="56" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H28))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -7570,12 +7763,46 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28">
-    <cfRule type="containsText" dxfId="40" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="55" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G28))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28">
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -8545,8 +8772,8 @@
       <c r="G36" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="21" t="s">
-        <v>0</v>
+      <c r="H36" s="38">
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -8567,8 +8794,8 @@
       <c r="G37" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H37" s="21" t="s">
-        <v>0</v>
+      <c r="H37" s="38">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -8580,11 +8807,28 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G33:H33 G35:H35 G3:H16 G19:H31">
-    <cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="54" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G33:H33 G35:H35 G3:H16 G19:H31">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18:H18">
+    <cfRule type="containsText" dxfId="53" priority="7" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18:H18">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -8596,12 +8840,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18:H18">
-    <cfRule type="containsText" dxfId="38" priority="3" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+  <conditionalFormatting sqref="G17:H17">
+    <cfRule type="containsText" dxfId="52" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G17))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18:H18">
+  <conditionalFormatting sqref="G17:H17">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -8613,12 +8874,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:H17">
-    <cfRule type="containsText" dxfId="37" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G17))))</formula>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:H17">
+  <conditionalFormatting sqref="H37">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -9617,8 +9878,8 @@
       <c r="G36" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H36" s="21" t="s">
-        <v>0</v>
+      <c r="H36" s="38">
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -9639,8 +9900,8 @@
       <c r="G37" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="H37" s="21" t="s">
-        <v>0</v>
+      <c r="H37" s="38">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9652,12 +9913,46 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G8:H31 G33:H33 G35:H35">
-    <cfRule type="containsText" dxfId="36" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="51" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G8))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G33:H33 G35:H35 G3:H31">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -9675,7 +9970,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="22" operator="containsText" text="*-" id="{4226227F-F842-4405-836A-DDD8E5CA33A1}">
+          <x14:cfRule type="containsText" priority="26" operator="containsText" text="*-" id="{4226227F-F842-4405-836A-DDD8E5CA33A1}">
             <xm:f>NOT(ISERROR(SEARCH(("*-"),('10копеек'!G3))))</xm:f>
             <x14:dxf>
               <fill>
@@ -10767,8 +11062,8 @@
       <c r="H37" s="1">
         <v>5</v>
       </c>
-      <c r="I37" s="1" t="s">
-        <v>0</v>
+      <c r="I37" s="38">
+        <v>1</v>
       </c>
       <c r="J37" s="10" t="str">
         <f t="shared" ref="J37:J38" si="4">IF(OR(AND(H37&gt;1,H37&lt;&gt;"-"),AND(I37&gt;1,I37&lt;&gt;"-")),"Can exchange","")</f>
@@ -10790,14 +11085,14 @@
       <c r="F38" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="G38" s="19" t="s">
-        <v>0</v>
+      <c r="G38" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="H38" s="1">
         <v>2</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>0</v>
+      <c r="I38" s="38">
+        <v>1</v>
       </c>
       <c r="J38" s="10" t="str">
         <f t="shared" si="4"/>
@@ -10813,10 +11108,10 @@
     <mergeCell ref="C1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:I32">
-    <cfRule type="containsText" dxfId="34" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="49" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="20">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -10827,11 +11122,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H33:I37">
-    <cfRule type="containsText" dxfId="33" priority="7" operator="containsText" text="*-">
+  <conditionalFormatting sqref="H33:I36 H37">
+    <cfRule type="containsText" dxfId="48" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -10842,10 +11137,44 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H38:I38">
-    <cfRule type="containsText" dxfId="32" priority="1" operator="containsText" text="*-">
+  <conditionalFormatting sqref="H38">
+    <cfRule type="containsText" dxfId="47" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H38))))</formula>
     </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
+    <cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I38">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I38))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I38">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -11867,14 +12196,14 @@
       <c r="E36" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F36" s="19" t="s">
-        <v>0</v>
+      <c r="F36" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="G36" s="1">
         <v>1</v>
       </c>
-      <c r="H36" s="1" t="s">
-        <v>0</v>
+      <c r="H36" s="38">
+        <v>1</v>
       </c>
       <c r="I36" s="10" t="str">
         <f t="shared" ref="I36:I37" si="3">IF(OR(AND(G36&gt;1,G36&lt;&gt;"-"),AND(H36&gt;1,H36&lt;&gt;"-")),"Can exchange","")</f>
@@ -11895,14 +12224,14 @@
       <c r="E37" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F37" s="19" t="s">
-        <v>0</v>
+      <c r="F37" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="G37" s="1">
         <v>2</v>
       </c>
-      <c r="H37" s="1" t="s">
-        <v>0</v>
+      <c r="H37" s="38">
+        <v>1</v>
       </c>
       <c r="I37" s="10" t="str">
         <f t="shared" si="3"/>
@@ -11918,6 +12247,43 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H30">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:H31">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:H31 G3:H7">
+    <cfRule type="containsText" dxfId="46" priority="13" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:H30">
+    <cfRule type="containsText" dxfId="45" priority="15" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G8))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32:H35 G37">
+    <cfRule type="containsText" dxfId="44" priority="11" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -11929,8 +12295,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G30:H31">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="G36">
+    <cfRule type="containsText" dxfId="43" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G36))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -11941,21 +12310,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G30:H31 G3:H7">
-    <cfRule type="containsText" dxfId="31" priority="9" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8:H30">
-    <cfRule type="containsText" dxfId="30" priority="11" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G8))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G32:H35 G37:H37">
-    <cfRule type="containsText" dxfId="29" priority="7" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="H36">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -11966,10 +12327,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G36:H36">
-    <cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G36))))</formula>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -13067,14 +13430,14 @@
       <c r="F37" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="G37" s="19" t="s">
-        <v>0</v>
+      <c r="G37" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="H37" s="1">
         <v>1</v>
       </c>
-      <c r="I37" s="1" t="s">
-        <v>0</v>
+      <c r="I37" s="38">
+        <v>1</v>
       </c>
       <c r="J37" s="10" t="str">
         <f t="shared" ref="J37" si="3">IF(OR(AND(H37&gt;1,H37&lt;&gt;"-"),AND(I37&gt;1,I37&lt;&gt;"-")),"Can exchange","")</f>
@@ -13096,14 +13459,14 @@
       <c r="F38" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="G38" s="19" t="s">
-        <v>0</v>
+      <c r="G38" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="H38" s="1">
         <v>2</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>0</v>
+      <c r="I38" s="38">
+        <v>1</v>
       </c>
       <c r="J38" s="10" t="str">
         <f t="shared" ref="J38" si="4">IF(OR(AND(H38&gt;1,H38&lt;&gt;"-"),AND(I38&gt;1,I38&lt;&gt;"-")),"Can exchange","")</f>
@@ -13119,7 +13482,7 @@
     <mergeCell ref="C1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="H9:I32">
-    <cfRule type="colorScale" priority="28">
+    <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -13131,11 +13494,26 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:I32">
-    <cfRule type="containsText" dxfId="27" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="42" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H8">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H33:I36 H37">
+    <cfRule type="containsText" dxfId="41" priority="21" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -13147,11 +13525,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H33:I37">
-    <cfRule type="containsText" dxfId="26" priority="17" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="containsText" dxfId="40" priority="15" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -13162,9 +13540,24 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3">
-    <cfRule type="containsText" dxfId="25" priority="11" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="containsText" dxfId="39" priority="13" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3">
+    <cfRule type="containsText" dxfId="38" priority="11" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
       <colorScale>
@@ -13177,24 +13570,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4">
-    <cfRule type="containsText" dxfId="24" priority="9" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3">
-    <cfRule type="containsText" dxfId="23" priority="7" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="containsText" dxfId="37" priority="7" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H38))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
       <colorScale>
@@ -13207,10 +13585,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H38:I38">
-    <cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H38))))</formula>
+  <conditionalFormatting sqref="I4:I8">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4:I8">
+    <cfRule type="containsText" dxfId="36" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I4))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -13222,7 +13619,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I8">
+  <conditionalFormatting sqref="I38">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I38))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I38">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -13234,11 +13636,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I8">
-    <cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(I4))))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -13246,7 +13643,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="21" operator="containsText" text="*-" id="{E9977262-0DF6-4236-8D1E-80CDB77D362D}">
+          <x14:cfRule type="containsText" priority="25" operator="containsText" text="*-" id="{E9977262-0DF6-4236-8D1E-80CDB77D362D}">
             <xm:f>NOT(ISERROR(SEARCH(("*-"),('10копеек'!H4))))</xm:f>
             <x14:dxf>
               <fill>
@@ -14310,8 +14707,8 @@
       <c r="H35" s="1">
         <v>1</v>
       </c>
-      <c r="I35" s="1" t="s">
-        <v>0</v>
+      <c r="I35" s="38">
+        <v>1</v>
       </c>
       <c r="J35" s="10" t="str">
         <f t="shared" ref="J35:J36" si="3">IF(OR(AND(H35&gt;1,H35&lt;&gt;"-"),AND(I35&gt;1,I35&lt;&gt;"-")),"Can exchange","")</f>
@@ -14322,27 +14719,25 @@
       <c r="A36" s="9">
         <v>2025</v>
       </c>
-      <c r="B36" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="G36" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>0</v>
+      <c r="B36" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
+      <c r="I36" s="38">
+        <v>1</v>
       </c>
       <c r="J36" s="10" t="str">
         <f t="shared" si="3"/>
@@ -14358,10 +14753,10 @@
     <mergeCell ref="C1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:I30">
-    <cfRule type="containsText" dxfId="19" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="34" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -14372,10 +14767,42 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31:I35">
-    <cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="*-">
+  <conditionalFormatting sqref="H31:I34 H35">
+    <cfRule type="containsText" dxfId="33" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
     </cfRule>
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="containsText" dxfId="32" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I35">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I35">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -14387,10 +14814,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H36:I36">
-    <cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H36))))</formula>
+  <conditionalFormatting sqref="I36">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(I36))))</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I36">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -15493,7 +15922,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H3 G4">
-    <cfRule type="containsText" dxfId="16" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="31" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -15508,7 +15937,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -15523,7 +15952,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:H36">
-    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="29" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G5))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">

</xml_diff>